<commit_message>
fixed - translations export: missing keys
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/21-producer-prns-check-selection.xlsx
+++ b/translations/welsh-translations/xlsx/21-producer-prns-check-selection.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="54">
   <si>
     <t>Translator notes</t>
   </si>
@@ -110,6 +110,69 @@
   </si>
   <si>
     <t>Action</t>
+  </si>
+  <si>
+    <t>prns.checkSelection.material.paper</t>
+  </si>
+  <si>
+    <t>Paper, board or fibre-based composite material</t>
+  </si>
+  <si>
+    <t>prns.checkSelection.material.plastic</t>
+  </si>
+  <si>
+    <t>Plastic</t>
+  </si>
+  <si>
+    <t>prns.checkSelection.material.wood</t>
+  </si>
+  <si>
+    <t>Wood</t>
+  </si>
+  <si>
+    <t>prns.checkSelection.material.steel</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>prns.checkSelection.material.aluminium</t>
+  </si>
+  <si>
+    <t>Aluminium</t>
+  </si>
+  <si>
+    <t>prns.checkSelection.material.glassOther</t>
+  </si>
+  <si>
+    <t>Glass Other</t>
+  </si>
+  <si>
+    <t>prns.checkSelection.material.glassRemelt</t>
+  </si>
+  <si>
+    <t>Glass Re-melt</t>
+  </si>
+  <si>
+    <t>prns.bulkConfirmation.material.paper</t>
+  </si>
+  <si>
+    <t>prns.bulkConfirmation.material.plastic</t>
+  </si>
+  <si>
+    <t>prns.bulkConfirmation.material.wood</t>
+  </si>
+  <si>
+    <t>prns.bulkConfirmation.material.steel</t>
+  </si>
+  <si>
+    <t>prns.bulkConfirmation.material.aluminium</t>
+  </si>
+  <si>
+    <t>prns.bulkConfirmation.material.glassOther</t>
+  </si>
+  <si>
+    <t>prns.bulkConfirmation.material.glassRemelt</t>
   </si>
 </sst>
 </file>
@@ -508,7 +571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -759,8 +822,288 @@
         <v>13</v>
       </c>
     </row>
+    <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F15"/>
+  <autoFilter ref="A5:F29"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>